<commit_message>
docs: atualiza readme e corrige formatação de moeda no main.py
</commit_message>
<xml_diff>
--- a/data/saida/candidatos_finalizados.xlsx
+++ b/data/saida/candidatos_finalizados.xlsx
@@ -480,8 +480,10 @@
       <c r="F2" t="n">
         <v>165</v>
       </c>
-      <c r="G2" t="n">
-        <v>4187.5</v>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>R$ 4.187,50</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -511,8 +513,10 @@
       <c r="F3" t="n">
         <v>160</v>
       </c>
-      <c r="G3" t="n">
-        <v>8000</v>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>R$ 8.000,00</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -542,8 +546,10 @@
       <c r="F4" t="n">
         <v>172</v>
       </c>
-      <c r="G4" t="n">
-        <v>14462.5</v>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>R$ 14.462,50</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -573,8 +579,10 @@
       <c r="F5" t="n">
         <v>160</v>
       </c>
-      <c r="G5" t="n">
-        <v>17000</v>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>R$ 17.000,00</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -604,8 +612,10 @@
       <c r="F6" t="n">
         <v>160</v>
       </c>
-      <c r="G6" t="n">
-        <v>8000</v>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>R$ 8.000,00</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -635,8 +645,10 @@
       <c r="F7" t="n">
         <v>180</v>
       </c>
-      <c r="G7" t="n">
-        <v>9500</v>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>R$ 9.500,00</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -666,8 +678,10 @@
       <c r="F8" t="n">
         <v>160</v>
       </c>
-      <c r="G8" t="n">
-        <v>13000</v>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>R$ 13.000,00</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -697,8 +711,10 @@
       <c r="F9" t="n">
         <v>162</v>
       </c>
-      <c r="G9" t="n">
-        <v>4075</v>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>R$ 4.075,00</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -728,8 +744,10 @@
       <c r="F10" t="n">
         <v>160</v>
       </c>
-      <c r="G10" t="n">
-        <v>8000</v>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>R$ 8.000,00</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -759,8 +777,10 @@
       <c r="F11" t="n">
         <v>160</v>
       </c>
-      <c r="G11" t="n">
-        <v>13000</v>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>R$ 13.000,00</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -790,8 +810,10 @@
       <c r="F12" t="n">
         <v>160</v>
       </c>
-      <c r="G12" t="n">
-        <v>4000</v>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>R$ 4.000,00</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -821,8 +843,10 @@
       <c r="F13" t="n">
         <v>164</v>
       </c>
-      <c r="G13" t="n">
-        <v>8300</v>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>R$ 8.300,00</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -852,8 +876,10 @@
       <c r="F14" t="n">
         <v>160</v>
       </c>
-      <c r="G14" t="n">
-        <v>8000</v>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>R$ 8.000,00</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -883,8 +909,10 @@
       <c r="F15" t="n">
         <v>168</v>
       </c>
-      <c r="G15" t="n">
-        <v>13975</v>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>R$ 13.975,00</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -914,8 +942,10 @@
       <c r="F16" t="n">
         <v>160</v>
       </c>
-      <c r="G16" t="n">
-        <v>17000</v>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>R$ 17.000,00</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -945,8 +975,10 @@
       <c r="F17" t="n">
         <v>170</v>
       </c>
-      <c r="G17" t="n">
-        <v>8750</v>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>R$ 8.750,00</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -976,8 +1008,10 @@
       <c r="F18" t="n">
         <v>160</v>
       </c>
-      <c r="G18" t="n">
-        <v>4000</v>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>R$ 4.000,00</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -1007,8 +1041,10 @@
       <c r="F19" t="n">
         <v>160</v>
       </c>
-      <c r="G19" t="n">
-        <v>8000</v>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>R$ 8.000,00</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -1038,8 +1074,10 @@
       <c r="F20" t="n">
         <v>160</v>
       </c>
-      <c r="G20" t="n">
-        <v>13000</v>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>R$ 13.000,00</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -1069,8 +1107,10 @@
       <c r="F21" t="n">
         <v>160</v>
       </c>
-      <c r="G21" t="n">
-        <v>4000</v>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>R$ 4.000,00</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -1100,8 +1140,10 @@
       <c r="F22" t="n">
         <v>178</v>
       </c>
-      <c r="G22" t="n">
-        <v>9350</v>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>R$ 9.350,00</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -1131,8 +1173,10 @@
       <c r="F23" t="n">
         <v>160</v>
       </c>
-      <c r="G23" t="n">
-        <v>13000</v>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>R$ 13.000,00</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -1162,8 +1206,10 @@
       <c r="F24" t="n">
         <v>160</v>
       </c>
-      <c r="G24" t="n">
-        <v>8000</v>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>R$ 8.000,00</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -1193,8 +1239,10 @@
       <c r="F25" t="n">
         <v>162</v>
       </c>
-      <c r="G25" t="n">
-        <v>8150</v>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>R$ 8.150,00</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -1224,8 +1272,10 @@
       <c r="F26" t="n">
         <v>160</v>
       </c>
-      <c r="G26" t="n">
-        <v>4000</v>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>R$ 4.000,00</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -1255,8 +1305,10 @@
       <c r="F27" t="n">
         <v>160</v>
       </c>
-      <c r="G27" t="n">
-        <v>8000</v>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>R$ 8.000,00</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -1286,8 +1338,10 @@
       <c r="F28" t="n">
         <v>185</v>
       </c>
-      <c r="G28" t="n">
-        <v>16046.88</v>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>R$ 16.046,88</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -1317,8 +1371,10 @@
       <c r="F29" t="n">
         <v>160</v>
       </c>
-      <c r="G29" t="n">
-        <v>8000</v>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>R$ 8.000,00</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -1348,8 +1404,10 @@
       <c r="F30" t="n">
         <v>160</v>
       </c>
-      <c r="G30" t="n">
-        <v>17000</v>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>R$ 17.000,00</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -1379,8 +1437,10 @@
       <c r="F31" t="n">
         <v>160</v>
       </c>
-      <c r="G31" t="n">
-        <v>4000</v>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>R$ 4.000,00</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -1410,8 +1470,10 @@
       <c r="F32" t="n">
         <v>170</v>
       </c>
-      <c r="G32" t="n">
-        <v>8750</v>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>R$ 8.750,00</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -1441,8 +1503,10 @@
       <c r="F33" t="n">
         <v>160</v>
       </c>
-      <c r="G33" t="n">
-        <v>8000</v>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>R$ 8.000,00</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -1472,8 +1536,10 @@
       <c r="F34" t="n">
         <v>160</v>
       </c>
-      <c r="G34" t="n">
-        <v>13000</v>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>R$ 13.000,00</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -1503,8 +1569,10 @@
       <c r="F35" t="n">
         <v>164</v>
       </c>
-      <c r="G35" t="n">
-        <v>4150</v>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>R$ 4.150,00</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -1534,8 +1602,10 @@
       <c r="F36" t="n">
         <v>160</v>
       </c>
-      <c r="G36" t="n">
-        <v>8000</v>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>R$ 8.000,00</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -1565,8 +1635,10 @@
       <c r="F37" t="n">
         <v>160</v>
       </c>
-      <c r="G37" t="n">
-        <v>8000</v>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>R$ 8.000,00</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -1596,8 +1668,10 @@
       <c r="F38" t="n">
         <v>160</v>
       </c>
-      <c r="G38" t="n">
-        <v>13000</v>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>R$ 13.000,00</t>
+        </is>
       </c>
     </row>
     <row r="39">
@@ -1627,8 +1701,10 @@
       <c r="F39" t="n">
         <v>160</v>
       </c>
-      <c r="G39" t="n">
-        <v>4000</v>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>R$ 4.000,00</t>
+        </is>
       </c>
     </row>
     <row r="40">
@@ -1658,8 +1734,10 @@
       <c r="F40" t="n">
         <v>160</v>
       </c>
-      <c r="G40" t="n">
-        <v>8000</v>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>R$ 8.000,00</t>
+        </is>
       </c>
     </row>
     <row r="41">
@@ -1689,8 +1767,10 @@
       <c r="F41" t="n">
         <v>160</v>
       </c>
-      <c r="G41" t="n">
-        <v>8000</v>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>R$ 8.000,00</t>
+        </is>
       </c>
     </row>
     <row r="42">
@@ -1720,8 +1800,10 @@
       <c r="F42" t="n">
         <v>160</v>
       </c>
-      <c r="G42" t="n">
-        <v>13000</v>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>R$ 13.000,00</t>
+        </is>
       </c>
     </row>
     <row r="43">
@@ -1751,8 +1833,10 @@
       <c r="F43" t="n">
         <v>160</v>
       </c>
-      <c r="G43" t="n">
-        <v>4000</v>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>R$ 4.000,00</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -1782,8 +1866,10 @@
       <c r="F44" t="n">
         <v>160</v>
       </c>
-      <c r="G44" t="n">
-        <v>8000</v>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>R$ 8.000,00</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -1813,8 +1899,10 @@
       <c r="F45" t="n">
         <v>172</v>
       </c>
-      <c r="G45" t="n">
-        <v>8900</v>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>R$ 8.900,00</t>
+        </is>
       </c>
     </row>
     <row r="46">
@@ -1844,8 +1932,10 @@
       <c r="F46" t="n">
         <v>160</v>
       </c>
-      <c r="G46" t="n">
-        <v>13000</v>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>R$ 13.000,00</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>